<commit_message>
Fix M5 regenerate date bug, replace PO auto-dedupe with warn-first flow, add per-column basket totals and skipped-SKU notice
</commit_message>
<xml_diff>
--- a/customers/cpall/excel_templates/versions/production_plan/v2.xlsx
+++ b/customers/cpall/excel_templates/versions/production_plan/v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ห้าง 7-11+ใบงาน\AUG 26\รอบเย็น\ทดสอบ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4FEB49-BD1B-471B-A1B9-98426802D90E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9121BC00-77DA-49A3-BB35-56CA18C5B451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="แพลน 7-11" sheetId="11" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'แพลน 7-11'!$C$5:$R$86</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'แพลน 7-11'!$C$5:$R$82</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="82">
   <si>
     <t>สุวรรณภูมิ</t>
   </si>
@@ -204,9 +204,6 @@
     <t>Kyoho Grape300gx 15 P</t>
   </si>
   <si>
-    <t>8859388008885    (ยอดเผื่อ)</t>
-  </si>
-  <si>
     <t>องุ่นไซน์มัสแคท 300 กรัม x 15 P</t>
   </si>
   <si>
@@ -214,12 +211,6 @@
   </si>
   <si>
     <t>8859388000018        (ยอดเผื่อ)</t>
-  </si>
-  <si>
-    <t>เชอร์รี่สดนำเข้า 150 กรัม x 36</t>
-  </si>
-  <si>
-    <t>Cherry150 g x 36 P  อเมริกา</t>
   </si>
   <si>
     <t>Red Seedless 150 g. x 32 P /     (จีน)</t>
@@ -1093,7 +1084,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="221">
+  <cellXfs count="215">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1524,6 +1515,201 @@
     <xf numFmtId="0" fontId="26" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="39" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1541,219 +1727,6 @@
     </xf>
     <xf numFmtId="3" fontId="30" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="31" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="34" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="34" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="34" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2110,7 +2083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C4:X108"/>
+  <dimension ref="C4:X104"/>
   <sheetFormatPr defaultColWidth="5.69921875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2.3984375" style="1" customWidth="1"/>
@@ -2140,150 +2113,150 @@
   <sheetData>
     <row r="4" spans="3:24" ht="15" customHeight="1" thickBot="1"/>
     <row r="5" spans="3:24" ht="15" customHeight="1">
-      <c r="C5" s="198"/>
-      <c r="D5" s="201" t="s">
+      <c r="C5" s="156"/>
+      <c r="D5" s="159" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="207" t="s">
+      <c r="E5" s="165" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="210" t="s">
+      <c r="F5" s="168" t="s">
         <v>1</v>
       </c>
-      <c r="G5" s="166" t="s">
-        <v>83</v>
-      </c>
-      <c r="H5" s="167"/>
-      <c r="I5" s="167"/>
-      <c r="J5" s="167"/>
-      <c r="K5" s="167"/>
-      <c r="L5" s="168"/>
-      <c r="M5" s="162" t="s">
-        <v>84</v>
-      </c>
-      <c r="N5" s="163"/>
-      <c r="O5" s="163"/>
-      <c r="P5" s="163"/>
-      <c r="Q5" s="163"/>
-      <c r="R5" s="147" t="s">
+      <c r="G5" s="177" t="s">
+        <v>80</v>
+      </c>
+      <c r="H5" s="178"/>
+      <c r="I5" s="178"/>
+      <c r="J5" s="178"/>
+      <c r="K5" s="178"/>
+      <c r="L5" s="179"/>
+      <c r="M5" s="173" t="s">
+        <v>81</v>
+      </c>
+      <c r="N5" s="174"/>
+      <c r="O5" s="174"/>
+      <c r="P5" s="174"/>
+      <c r="Q5" s="174"/>
+      <c r="R5" s="212" t="s">
         <v>3</v>
       </c>
-      <c r="S5" s="144" t="s">
+      <c r="S5" s="209" t="s">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
     </row>
     <row r="6" spans="3:24" ht="73.2" customHeight="1" thickBot="1">
-      <c r="C6" s="199"/>
-      <c r="D6" s="202"/>
-      <c r="E6" s="208"/>
-      <c r="F6" s="211"/>
-      <c r="G6" s="169"/>
-      <c r="H6" s="170"/>
-      <c r="I6" s="170"/>
-      <c r="J6" s="170"/>
-      <c r="K6" s="170"/>
-      <c r="L6" s="171"/>
-      <c r="M6" s="164"/>
-      <c r="N6" s="165"/>
-      <c r="O6" s="165"/>
-      <c r="P6" s="165"/>
-      <c r="Q6" s="165"/>
-      <c r="R6" s="148"/>
-      <c r="S6" s="145"/>
+      <c r="C6" s="157"/>
+      <c r="D6" s="160"/>
+      <c r="E6" s="166"/>
+      <c r="F6" s="169"/>
+      <c r="G6" s="180"/>
+      <c r="H6" s="181"/>
+      <c r="I6" s="181"/>
+      <c r="J6" s="181"/>
+      <c r="K6" s="181"/>
+      <c r="L6" s="182"/>
+      <c r="M6" s="175"/>
+      <c r="N6" s="176"/>
+      <c r="O6" s="176"/>
+      <c r="P6" s="176"/>
+      <c r="Q6" s="176"/>
+      <c r="R6" s="213"/>
+      <c r="S6" s="210"/>
       <c r="X6" s="1"/>
     </row>
     <row r="7" spans="3:24" ht="55.2" customHeight="1" thickBot="1">
-      <c r="C7" s="199"/>
-      <c r="D7" s="202"/>
-      <c r="E7" s="208"/>
-      <c r="F7" s="211"/>
-      <c r="G7" s="172" t="s">
+      <c r="C7" s="157"/>
+      <c r="D7" s="160"/>
+      <c r="E7" s="166"/>
+      <c r="F7" s="169"/>
+      <c r="G7" s="183" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="175" t="s">
+      <c r="H7" s="186" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="176"/>
-      <c r="J7" s="177"/>
-      <c r="K7" s="182" t="s">
+      <c r="I7" s="187"/>
+      <c r="J7" s="188"/>
+      <c r="K7" s="193" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="185" t="s">
+      <c r="L7" s="196" t="s">
         <v>0</v>
       </c>
-      <c r="M7" s="194" t="s">
+      <c r="M7" s="205" t="s">
         <v>23</v>
       </c>
-      <c r="N7" s="195"/>
-      <c r="O7" s="195"/>
-      <c r="P7" s="195"/>
-      <c r="Q7" s="195"/>
-      <c r="R7" s="148"/>
-      <c r="S7" s="145"/>
+      <c r="N7" s="206"/>
+      <c r="O7" s="206"/>
+      <c r="P7" s="206"/>
+      <c r="Q7" s="206"/>
+      <c r="R7" s="213"/>
+      <c r="S7" s="210"/>
       <c r="X7" s="1"/>
     </row>
     <row r="8" spans="3:24" ht="68.400000000000006" customHeight="1">
-      <c r="C8" s="199"/>
-      <c r="D8" s="202"/>
-      <c r="E8" s="208"/>
-      <c r="F8" s="211"/>
-      <c r="G8" s="173"/>
-      <c r="H8" s="180" t="s">
+      <c r="C8" s="157"/>
+      <c r="D8" s="160"/>
+      <c r="E8" s="166"/>
+      <c r="F8" s="169"/>
+      <c r="G8" s="184"/>
+      <c r="H8" s="191" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="178" t="s">
+      <c r="I8" s="189" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="178" t="s">
+      <c r="J8" s="189" t="s">
         <v>24</v>
       </c>
-      <c r="K8" s="183"/>
-      <c r="L8" s="186"/>
-      <c r="M8" s="196" t="s">
+      <c r="K8" s="194"/>
+      <c r="L8" s="197"/>
+      <c r="M8" s="207" t="s">
         <v>4</v>
       </c>
-      <c r="N8" s="196" t="s">
+      <c r="N8" s="207" t="s">
         <v>49</v>
       </c>
-      <c r="O8" s="188" t="s">
+      <c r="O8" s="199" t="s">
         <v>5</v>
       </c>
-      <c r="P8" s="190" t="s">
+      <c r="P8" s="201" t="s">
         <v>6</v>
       </c>
-      <c r="Q8" s="192" t="s">
+      <c r="Q8" s="203" t="s">
         <v>7</v>
       </c>
-      <c r="R8" s="148"/>
-      <c r="S8" s="145"/>
+      <c r="R8" s="213"/>
+      <c r="S8" s="210"/>
       <c r="X8" s="1"/>
     </row>
     <row r="9" spans="3:24" ht="18" customHeight="1" thickBot="1">
-      <c r="C9" s="199"/>
-      <c r="D9" s="202"/>
-      <c r="E9" s="208"/>
-      <c r="F9" s="211"/>
-      <c r="G9" s="174"/>
-      <c r="H9" s="181"/>
-      <c r="I9" s="179"/>
-      <c r="J9" s="179"/>
-      <c r="K9" s="184"/>
-      <c r="L9" s="187"/>
-      <c r="M9" s="197"/>
-      <c r="N9" s="197"/>
-      <c r="O9" s="189"/>
-      <c r="P9" s="191"/>
-      <c r="Q9" s="193"/>
-      <c r="R9" s="149"/>
-      <c r="S9" s="145"/>
+      <c r="C9" s="157"/>
+      <c r="D9" s="160"/>
+      <c r="E9" s="166"/>
+      <c r="F9" s="169"/>
+      <c r="G9" s="185"/>
+      <c r="H9" s="192"/>
+      <c r="I9" s="190"/>
+      <c r="J9" s="190"/>
+      <c r="K9" s="195"/>
+      <c r="L9" s="198"/>
+      <c r="M9" s="208"/>
+      <c r="N9" s="208"/>
+      <c r="O9" s="200"/>
+      <c r="P9" s="202"/>
+      <c r="Q9" s="204"/>
+      <c r="R9" s="214"/>
+      <c r="S9" s="210"/>
       <c r="X9" s="1"/>
     </row>
     <row r="10" spans="3:24" ht="67.95" customHeight="1" thickBot="1">
-      <c r="C10" s="200"/>
-      <c r="D10" s="203"/>
-      <c r="E10" s="209"/>
-      <c r="F10" s="211"/>
+      <c r="C10" s="158"/>
+      <c r="D10" s="161"/>
+      <c r="E10" s="167"/>
+      <c r="F10" s="169"/>
       <c r="G10" s="50" t="s">
         <v>16</v>
       </c>
@@ -2320,20 +2293,20 @@
       <c r="R10" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="S10" s="146"/>
+      <c r="S10" s="211"/>
       <c r="X10" s="1"/>
     </row>
     <row r="11" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C11" s="150">
+      <c r="C11" s="162">
         <v>1</v>
       </c>
       <c r="D11" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="215">
+      <c r="E11" s="170">
         <v>21.5</v>
       </c>
-      <c r="F11" s="156">
+      <c r="F11" s="153">
         <v>36</v>
       </c>
       <c r="G11" s="84"/>
@@ -2357,12 +2330,12 @@
       <c r="X11" s="1"/>
     </row>
     <row r="12" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C12" s="151"/>
+      <c r="C12" s="163"/>
       <c r="D12" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="216"/>
-      <c r="F12" s="157"/>
+      <c r="E12" s="171"/>
+      <c r="F12" s="154"/>
       <c r="G12" s="89" t="str">
         <f>IF(G11=0, "", IF(MOD(G11, $F$11) = 0, G11 / $F$11, IF(INT(G11 / $F$11) = 0, MOD(G11, $F$11) &amp; " P", INT(G11 / $F$11) &amp; " + " &amp; MOD(G11, $F$11) &amp; " P")))</f>
         <v/>
@@ -2419,12 +2392,12 @@
       <c r="X12" s="1"/>
     </row>
     <row r="13" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C13" s="151"/>
+      <c r="C13" s="163"/>
       <c r="D13" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="216"/>
-      <c r="F13" s="157"/>
+      <c r="E13" s="171"/>
+      <c r="F13" s="154"/>
       <c r="G13" s="94"/>
       <c r="H13" s="95"/>
       <c r="I13" s="96"/>
@@ -2444,12 +2417,12 @@
       <c r="X13" s="1"/>
     </row>
     <row r="14" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C14" s="152"/>
+      <c r="C14" s="164"/>
       <c r="D14" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="217"/>
-      <c r="F14" s="158"/>
+      <c r="E14" s="172"/>
+      <c r="F14" s="155"/>
       <c r="G14" s="103"/>
       <c r="H14" s="104"/>
       <c r="I14" s="105"/>
@@ -2470,16 +2443,16 @@
       <c r="X14" s="1"/>
     </row>
     <row r="15" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C15" s="150">
+      <c r="C15" s="162">
         <v>2</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="218">
+      <c r="E15" s="144">
         <v>24</v>
       </c>
-      <c r="F15" s="156">
+      <c r="F15" s="153">
         <v>32</v>
       </c>
       <c r="G15" s="84"/>
@@ -2503,12 +2476,12 @@
       <c r="X15" s="1"/>
     </row>
     <row r="16" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C16" s="151"/>
+      <c r="C16" s="163"/>
       <c r="D16" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="219"/>
-      <c r="F16" s="157"/>
+      <c r="E16" s="145"/>
+      <c r="F16" s="154"/>
       <c r="G16" s="89" t="str">
         <f>IF(G15=0, "", IF(MOD(G15, $F$15) = 0, G15 / $F$15, IF(INT(G15 / $F$15) = 0, MOD(G15, $F$15) &amp; " P", INT(G15 / $F$15) &amp; " + " &amp; MOD(G15, $F$15) &amp; " P")))</f>
         <v/>
@@ -2565,12 +2538,12 @@
       <c r="X16" s="1"/>
     </row>
     <row r="17" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C17" s="151"/>
+      <c r="C17" s="163"/>
       <c r="D17" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="219"/>
-      <c r="F17" s="157"/>
+      <c r="E17" s="145"/>
+      <c r="F17" s="154"/>
       <c r="G17" s="94"/>
       <c r="H17" s="95"/>
       <c r="I17" s="96"/>
@@ -2590,12 +2563,12 @@
       <c r="X17" s="1"/>
     </row>
     <row r="18" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C18" s="152"/>
+      <c r="C18" s="164"/>
       <c r="D18" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E18" s="219"/>
-      <c r="F18" s="157"/>
+      <c r="E18" s="145"/>
+      <c r="F18" s="154"/>
       <c r="G18" s="115"/>
       <c r="H18" s="116"/>
       <c r="I18" s="117"/>
@@ -2616,19 +2589,19 @@
       <c r="X18" s="1"/>
     </row>
     <row r="19" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C19" s="204">
-        <v>3</v>
+      <c r="C19" s="74">
+        <v>4</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="E19" s="212">
-        <v>64</v>
-      </c>
-      <c r="F19" s="156">
-        <v>36</v>
-      </c>
-      <c r="G19" s="84"/>
+        <v>73</v>
+      </c>
+      <c r="E19" s="144">
+        <v>43</v>
+      </c>
+      <c r="F19" s="147">
+        <v>14</v>
+      </c>
+      <c r="G19" s="86"/>
       <c r="H19" s="85"/>
       <c r="I19" s="85"/>
       <c r="J19" s="85"/>
@@ -2643,24 +2616,22 @@
         <f>SUM(G19:Q19)</f>
         <v>0</v>
       </c>
-      <c r="S19" s="37" t="s">
+      <c r="S19" s="38" t="s">
         <v>19</v>
       </c>
       <c r="X19" s="1"/>
     </row>
     <row r="20" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C20" s="205"/>
-      <c r="D20" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E20" s="213"/>
-      <c r="F20" s="157"/>
-      <c r="G20" s="89" t="str">
-        <f t="shared" ref="G20:Q20" si="2">IF(G19=0, "", IF(MOD(G19, $F$19) = 0, G19/ $F$19, IF(INT(G19 / $F$19) = 0, MOD(G19, $F$19) &amp; " P", INT(G19 / $F$19) &amp; " + " &amp; MOD(G19, $F$19) &amp; " P")))</f>
+      <c r="C20" s="76"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="145"/>
+      <c r="F20" s="148"/>
+      <c r="G20" s="91" t="str">
+        <f>IF(G19=0, "", IF(MOD(G19, $F$19) = 0, G19/ $F$19, IF(INT(G19 / $F$19) = 0, MOD(G19, $F$19) &amp; " P", INT(G19 / $F$19) &amp; " + " &amp; MOD(G19, $F$19) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H20" s="90" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="H20:Q20" si="2">IF(H19=0, "", IF(MOD(H19, $F$19) = 0, H19/ $F$19, IF(INT(H19 / $F$19) = 0, MOD(H19, $F$19) &amp; " P", INT(H19 / $F$19) &amp; " + " &amp; MOD(H19, $F$19) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I20" s="90" t="str">
@@ -2701,22 +2672,22 @@
       </c>
       <c r="R20" s="138">
         <f>G19+H19+I19+J19+K19+L19+O21</f>
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="S20" s="141">
-        <f>SUM(O22)</f>
-        <v>280</v>
+        <f>O22</f>
+        <v>200</v>
       </c>
       <c r="X20" s="1"/>
     </row>
     <row r="21" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C21" s="205"/>
-      <c r="D21" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="213"/>
-      <c r="F21" s="157"/>
-      <c r="G21" s="94"/>
+      <c r="C21" s="76"/>
+      <c r="D21" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" s="145"/>
+      <c r="F21" s="148"/>
+      <c r="G21" s="112"/>
       <c r="H21" s="95"/>
       <c r="I21" s="96"/>
       <c r="J21" s="97"/>
@@ -2725,7 +2696,7 @@
       <c r="M21" s="100"/>
       <c r="N21" s="100"/>
       <c r="O21" s="102">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="P21" s="100"/>
       <c r="Q21" s="113"/>
@@ -2734,41 +2705,41 @@
       <c r="X21" s="1"/>
     </row>
     <row r="22" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C22" s="206"/>
+      <c r="C22" s="77"/>
       <c r="D22" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E22" s="214"/>
-      <c r="F22" s="158"/>
+      <c r="E22" s="146"/>
+      <c r="F22" s="149"/>
       <c r="G22" s="125"/>
-      <c r="H22" s="104"/>
-      <c r="I22" s="105"/>
-      <c r="J22" s="106"/>
+      <c r="H22" s="116"/>
+      <c r="I22" s="117"/>
+      <c r="J22" s="118"/>
       <c r="K22" s="108"/>
-      <c r="L22" s="125"/>
+      <c r="L22" s="120"/>
       <c r="M22" s="109"/>
       <c r="N22" s="109"/>
       <c r="O22" s="111">
         <f>SUM(O21-M19-N19-O19-P19-Q19)</f>
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="P22" s="109"/>
       <c r="Q22" s="126"/>
       <c r="R22" s="140"/>
-      <c r="S22" s="143"/>
+      <c r="S22" s="142"/>
       <c r="X22" s="1"/>
     </row>
     <row r="23" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C23" s="74">
-        <v>4</v>
+      <c r="C23" s="75">
+        <v>5</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="E23" s="218">
-        <v>43</v>
-      </c>
-      <c r="F23" s="159">
+        <v>75</v>
+      </c>
+      <c r="E23" s="150">
+        <v>38</v>
+      </c>
+      <c r="F23" s="153">
         <v>14</v>
       </c>
       <c r="G23" s="86"/>
@@ -2793,9 +2764,9 @@
     </row>
     <row r="24" spans="3:24" ht="67.5" customHeight="1">
       <c r="C24" s="76"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="219"/>
-      <c r="F24" s="160"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="151"/>
+      <c r="F24" s="154"/>
       <c r="G24" s="91" t="str">
         <f>IF(G23=0, "", IF(MOD(G23, $F$23) = 0, G23/ $F$23, IF(INT(G23 / $F$23) = 0, MOD(G23, $F$23) &amp; " P", INT(G23 / $F$23) &amp; " + " &amp; MOD(G23, $F$23) &amp; " P")))</f>
         <v/>
@@ -2852,11 +2823,11 @@
     </row>
     <row r="25" spans="3:24" ht="67.5" customHeight="1">
       <c r="C25" s="76"/>
-      <c r="D25" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" s="219"/>
-      <c r="F25" s="160"/>
+      <c r="D25" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E25" s="151"/>
+      <c r="F25" s="154"/>
       <c r="G25" s="112"/>
       <c r="H25" s="95"/>
       <c r="I25" s="96"/>
@@ -2879,8 +2850,8 @@
       <c r="D26" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E26" s="220"/>
-      <c r="F26" s="161"/>
+      <c r="E26" s="152"/>
+      <c r="F26" s="155"/>
       <c r="G26" s="125"/>
       <c r="H26" s="116"/>
       <c r="I26" s="117"/>
@@ -2900,17 +2871,17 @@
       <c r="X26" s="1"/>
     </row>
     <row r="27" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C27" s="75">
-        <v>5</v>
+      <c r="C27" s="162">
+        <v>6</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" s="153">
-        <v>38</v>
-      </c>
-      <c r="F27" s="156">
-        <v>14</v>
+        <v>59</v>
+      </c>
+      <c r="E27" s="150">
+        <v>21.5</v>
+      </c>
+      <c r="F27" s="153">
+        <v>32</v>
       </c>
       <c r="G27" s="86"/>
       <c r="H27" s="85"/>
@@ -2933,10 +2904,12 @@
       <c r="X27" s="1"/>
     </row>
     <row r="28" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C28" s="76"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="154"/>
-      <c r="F28" s="157"/>
+      <c r="C28" s="163"/>
+      <c r="D28" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E28" s="151"/>
+      <c r="F28" s="154"/>
       <c r="G28" s="91" t="str">
         <f>IF(G27=0, "", IF(MOD(G27, $F$27) = 0, G27/ $F$27, IF(INT(G27 / $F$27) = 0, MOD(G27, $F$27) &amp; " P", INT(G27 / $F$27) &amp; " + " &amp; MOD(G27, $F$27) &amp; " P")))</f>
         <v/>
@@ -2983,21 +2956,21 @@
       </c>
       <c r="R28" s="138">
         <f>G27+H27+I27+J27+K27+L27+O29</f>
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="S28" s="141">
         <f>O30</f>
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="X28" s="1"/>
     </row>
     <row r="29" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C29" s="76"/>
-      <c r="D29" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="E29" s="154"/>
-      <c r="F29" s="157"/>
+      <c r="C29" s="163"/>
+      <c r="D29" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E29" s="151"/>
+      <c r="F29" s="154"/>
       <c r="G29" s="112"/>
       <c r="H29" s="95"/>
       <c r="I29" s="96"/>
@@ -3007,7 +2980,7 @@
       <c r="M29" s="100"/>
       <c r="N29" s="100"/>
       <c r="O29" s="102">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="P29" s="100"/>
       <c r="Q29" s="113"/>
@@ -3016,12 +2989,12 @@
       <c r="X29" s="1"/>
     </row>
     <row r="30" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C30" s="77"/>
+      <c r="C30" s="164"/>
       <c r="D30" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E30" s="155"/>
-      <c r="F30" s="158"/>
+      <c r="E30" s="152"/>
+      <c r="F30" s="155"/>
       <c r="G30" s="125"/>
       <c r="H30" s="116"/>
       <c r="I30" s="117"/>
@@ -3032,7 +3005,7 @@
       <c r="N30" s="109"/>
       <c r="O30" s="111">
         <f>SUM(O29-M27-N27-O27-P27-Q27)</f>
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="P30" s="109"/>
       <c r="Q30" s="126"/>
@@ -3041,17 +3014,17 @@
       <c r="X30" s="1"/>
     </row>
     <row r="31" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C31" s="150">
-        <v>6</v>
+      <c r="C31" s="39">
+        <v>7</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="E31" s="153">
-        <v>21.5</v>
-      </c>
-      <c r="F31" s="156">
-        <v>32</v>
+        <v>66</v>
+      </c>
+      <c r="E31" s="150">
+        <v>33</v>
+      </c>
+      <c r="F31" s="153">
+        <v>27</v>
       </c>
       <c r="G31" s="86"/>
       <c r="H31" s="85"/>
@@ -3074,12 +3047,12 @@
       <c r="X31" s="1"/>
     </row>
     <row r="32" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C32" s="151"/>
-      <c r="D32" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="E32" s="154"/>
-      <c r="F32" s="157"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="151"/>
+      <c r="F32" s="154"/>
       <c r="G32" s="91" t="str">
         <f>IF(G31=0, "", IF(MOD(G31, $F$31) = 0, G31/ $F$31, IF(INT(G31 / $F$31) = 0, MOD(G31, $F$31) &amp; " P", INT(G31 / $F$31) &amp; " + " &amp; MOD(G31, $F$31) &amp; " P")))</f>
         <v/>
@@ -3126,21 +3099,21 @@
       </c>
       <c r="R32" s="138">
         <f>G31+H31+I31+J31+K31+L31+O33</f>
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="S32" s="141">
         <f>O34</f>
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="X32" s="1"/>
     </row>
     <row r="33" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C33" s="151"/>
-      <c r="D33" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="E33" s="154"/>
-      <c r="F33" s="157"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="E33" s="151"/>
+      <c r="F33" s="154"/>
       <c r="G33" s="112"/>
       <c r="H33" s="95"/>
       <c r="I33" s="96"/>
@@ -3150,7 +3123,7 @@
       <c r="M33" s="100"/>
       <c r="N33" s="100"/>
       <c r="O33" s="102">
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="P33" s="100"/>
       <c r="Q33" s="113"/>
@@ -3159,12 +3132,12 @@
       <c r="X33" s="1"/>
     </row>
     <row r="34" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C34" s="152"/>
+      <c r="C34" s="41"/>
       <c r="D34" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E34" s="155"/>
-      <c r="F34" s="158"/>
+      <c r="E34" s="152"/>
+      <c r="F34" s="155"/>
       <c r="G34" s="125"/>
       <c r="H34" s="116"/>
       <c r="I34" s="117"/>
@@ -3175,7 +3148,7 @@
       <c r="N34" s="109"/>
       <c r="O34" s="111">
         <f>SUM(O33-M31-N31-O31-P31-Q31)</f>
-        <v>350</v>
+        <v>0</v>
       </c>
       <c r="P34" s="109"/>
       <c r="Q34" s="126"/>
@@ -3184,24 +3157,24 @@
       <c r="X34" s="1"/>
     </row>
     <row r="35" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C35" s="39">
-        <v>7</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="E35" s="153">
-        <v>33</v>
-      </c>
-      <c r="F35" s="156">
+      <c r="C35" s="63">
+        <v>8</v>
+      </c>
+      <c r="D35" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="E35" s="66">
+        <v>125</v>
+      </c>
+      <c r="F35" s="147">
         <v>27</v>
       </c>
       <c r="G35" s="86"/>
       <c r="H35" s="85"/>
       <c r="I35" s="85"/>
       <c r="J35" s="85"/>
-      <c r="K35" s="86"/>
-      <c r="L35" s="86"/>
+      <c r="K35" s="84"/>
+      <c r="L35" s="127"/>
       <c r="M35" s="86"/>
       <c r="N35" s="86"/>
       <c r="O35" s="86"/>
@@ -3211,36 +3184,36 @@
         <f>SUM(G35:Q35)</f>
         <v>0</v>
       </c>
-      <c r="S35" s="38" t="s">
+      <c r="S35" s="37" t="s">
         <v>19</v>
       </c>
       <c r="X35" s="1"/>
     </row>
     <row r="36" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C36" s="40"/>
-      <c r="D36" s="43" t="s">
-        <v>71</v>
-      </c>
-      <c r="E36" s="154"/>
-      <c r="F36" s="157"/>
+      <c r="C36" s="64"/>
+      <c r="D36" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E36" s="67"/>
+      <c r="F36" s="148"/>
       <c r="G36" s="91" t="str">
         <f>IF(G35=0, "", IF(MOD(G35, $F$35) = 0, G35/ $F$35, IF(INT(G35 / $F$35) = 0, MOD(G35, $F$35) &amp; " P", INT(G35 / $F$35) &amp; " + " &amp; MOD(G35, $F$35) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H36" s="90" t="str">
-        <f t="shared" ref="H36:Q36" si="6">IF(H35=0, "", IF(MOD(H35, $F$35) = 0, H35/ $F$35, IF(INT(H35 / $F$35) = 0, MOD(H35, $F$35) &amp; " P", INT(H35 / $F$35) &amp; " + " &amp; MOD(H35, $F$35) &amp; " P")))</f>
+        <f>IF(H35=0, "", IF(MOD(H35, $F$35) = 0, H35/ $F$35, IF(INT(H35 / $F$35) = 0, MOD(H35, $F$35) &amp; " P", INT(H35 / $F$35) &amp; " + " &amp; MOD(H35, $F$35) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I36" s="90" t="str">
-        <f t="shared" si="6"/>
+        <f>IF(I35=0, "", IF(MOD(I35, $F$35) = 0, I35/ $F$35, IF(INT(I35 / $F$35) = 0, MOD(I35, $F$35) &amp; " P", INT(I35 / $F$35) &amp; " + " &amp; MOD(I35, $F$35) &amp; " P")))</f>
         <v/>
       </c>
       <c r="J36" s="90" t="str">
-        <f t="shared" si="6"/>
+        <f>IF(J35=0, "", IF(MOD(J35, $F$35) = 0, J35/ $F$35, IF(INT(J35 / $F$35) = 0, MOD(J35, $F$35) &amp; " P", INT(J35 / $F$35) &amp; " + " &amp; MOD(J35, $F$35) &amp; " P")))</f>
         <v/>
       </c>
       <c r="K36" s="91" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="K36:Q36" si="6">IF(K35=0, "", IF(MOD(K35, $F$35) = 0, K35/ $F$35, IF(INT(K35 / $F$35) = 0, MOD(K35, $F$35) &amp; " P", INT(K35 / $F$35) &amp; " + " &amp; MOD(K35, $F$35) &amp; " P")))</f>
         <v/>
       </c>
       <c r="L36" s="91" t="str">
@@ -3269,21 +3242,21 @@
       </c>
       <c r="R36" s="138">
         <f>G35+H35+I35+J35+K35+L35+O37</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="S36" s="141">
         <f>O38</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="X36" s="1"/>
     </row>
     <row r="37" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C37" s="40"/>
-      <c r="D37" s="42" t="s">
+      <c r="C37" s="64"/>
+      <c r="D37" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E37" s="154"/>
-      <c r="F37" s="157"/>
+      <c r="E37" s="67"/>
+      <c r="F37" s="148"/>
       <c r="G37" s="112"/>
       <c r="H37" s="95"/>
       <c r="I37" s="96"/>
@@ -3293,7 +3266,7 @@
       <c r="M37" s="100"/>
       <c r="N37" s="100"/>
       <c r="O37" s="102">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="P37" s="100"/>
       <c r="Q37" s="113"/>
@@ -3302,42 +3275,42 @@
       <c r="X37" s="1"/>
     </row>
     <row r="38" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C38" s="41"/>
-      <c r="D38" s="14" t="s">
+      <c r="C38" s="65"/>
+      <c r="D38" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E38" s="155"/>
-      <c r="F38" s="158"/>
-      <c r="G38" s="125"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="149"/>
+      <c r="G38" s="120"/>
       <c r="H38" s="116"/>
       <c r="I38" s="117"/>
       <c r="J38" s="118"/>
-      <c r="K38" s="108"/>
+      <c r="K38" s="119"/>
       <c r="L38" s="120"/>
-      <c r="M38" s="109"/>
-      <c r="N38" s="109"/>
+      <c r="M38" s="128"/>
+      <c r="N38" s="128"/>
       <c r="O38" s="111">
         <f>SUM(O37-M35-N35-O35-P35-Q35)</f>
-        <v>0</v>
-      </c>
-      <c r="P38" s="109"/>
-      <c r="Q38" s="126"/>
+        <v>250</v>
+      </c>
+      <c r="P38" s="128"/>
+      <c r="Q38" s="121"/>
       <c r="R38" s="140"/>
       <c r="S38" s="142"/>
       <c r="X38" s="1"/>
     </row>
     <row r="39" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C39" s="63">
-        <v>8</v>
+      <c r="C39" s="59">
+        <v>9</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="E39" s="66">
-        <v>125</v>
-      </c>
-      <c r="F39" s="159">
-        <v>27</v>
+        <v>69</v>
+      </c>
+      <c r="E39" s="24">
+        <v>55</v>
+      </c>
+      <c r="F39" s="44">
+        <v>36</v>
       </c>
       <c r="G39" s="86"/>
       <c r="H39" s="85"/>
@@ -3360,30 +3333,30 @@
       <c r="X39" s="1"/>
     </row>
     <row r="40" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C40" s="64"/>
+      <c r="C40" s="60"/>
       <c r="D40" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E40" s="67"/>
-      <c r="F40" s="160"/>
+        <v>29</v>
+      </c>
+      <c r="E40" s="25"/>
+      <c r="F40" s="45"/>
       <c r="G40" s="91" t="str">
         <f>IF(G39=0, "", IF(MOD(G39, $F$39) = 0, G39/ $F$39, IF(INT(G39 / $F$39) = 0, MOD(G39, $F$39) &amp; " P", INT(G39 / $F$39) &amp; " + " &amp; MOD(G39, $F$39) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H40" s="90" t="str">
-        <f>IF(H39=0, "", IF(MOD(H39, $F$39) = 0, H39/ $F$39, IF(INT(H39 / $F$39) = 0, MOD(H39, $F$39) &amp; " P", INT(H39 / $F$39) &amp; " + " &amp; MOD(H39, $F$39) &amp; " P")))</f>
+        <f t="shared" ref="H40:Q40" si="7">IF(H39=0, "", IF(MOD(H39, $F$39) = 0, H39/ $F$39, IF(INT(H39 / $F$39) = 0, MOD(H39, $F$39) &amp; " P", INT(H39 / $F$39) &amp; " + " &amp; MOD(H39, $F$39) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I40" s="90" t="str">
-        <f>IF(I39=0, "", IF(MOD(I39, $F$39) = 0, I39/ $F$39, IF(INT(I39 / $F$39) = 0, MOD(I39, $F$39) &amp; " P", INT(I39 / $F$39) &amp; " + " &amp; MOD(I39, $F$39) &amp; " P")))</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="J40" s="90" t="str">
-        <f>IF(J39=0, "", IF(MOD(J39, $F$39) = 0, J39/ $F$39, IF(INT(J39 / $F$39) = 0, MOD(J39, $F$39) &amp; " P", INT(J39 / $F$39) &amp; " + " &amp; MOD(J39, $F$39) &amp; " P")))</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="K40" s="91" t="str">
-        <f t="shared" ref="K40:Q40" si="7">IF(K39=0, "", IF(MOD(K39, $F$39) = 0, K39/ $F$39, IF(INT(K39 / $F$39) = 0, MOD(K39, $F$39) &amp; " P", INT(K39 / $F$39) &amp; " + " &amp; MOD(K39, $F$39) &amp; " P")))</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="L40" s="91" t="str">
@@ -3412,21 +3385,21 @@
       </c>
       <c r="R40" s="138">
         <f>G39+H39+I39+J39+K39+L39+O41</f>
-        <v>250</v>
+        <v>650</v>
       </c>
       <c r="S40" s="141">
         <f>O42</f>
-        <v>250</v>
+        <v>650</v>
       </c>
       <c r="X40" s="1"/>
     </row>
     <row r="41" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C41" s="64"/>
+      <c r="C41" s="60"/>
       <c r="D41" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E41" s="67"/>
-      <c r="F41" s="160"/>
+        <v>33</v>
+      </c>
+      <c r="E41" s="25"/>
+      <c r="F41" s="45"/>
       <c r="G41" s="112"/>
       <c r="H41" s="95"/>
       <c r="I41" s="96"/>
@@ -3436,7 +3409,7 @@
       <c r="M41" s="100"/>
       <c r="N41" s="100"/>
       <c r="O41" s="102">
-        <v>250</v>
+        <v>650</v>
       </c>
       <c r="P41" s="100"/>
       <c r="Q41" s="113"/>
@@ -3445,12 +3418,12 @@
       <c r="X41" s="1"/>
     </row>
     <row r="42" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C42" s="65"/>
+      <c r="C42" s="61"/>
       <c r="D42" s="8" t="s">
         <v>8</v>
       </c>
       <c r="E42" s="26"/>
-      <c r="F42" s="161"/>
+      <c r="F42" s="46"/>
       <c r="G42" s="120"/>
       <c r="H42" s="116"/>
       <c r="I42" s="117"/>
@@ -3461,7 +3434,7 @@
       <c r="N42" s="128"/>
       <c r="O42" s="111">
         <f>SUM(O41-M39-N39-O39-P39-Q39)</f>
-        <v>250</v>
+        <v>650</v>
       </c>
       <c r="P42" s="128"/>
       <c r="Q42" s="121"/>
@@ -3471,28 +3444,28 @@
     </row>
     <row r="43" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C43" s="59">
-        <v>9</v>
-      </c>
-      <c r="D43" s="22" t="s">
-        <v>72</v>
+        <v>10</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>39</v>
       </c>
       <c r="E43" s="24">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="F43" s="44">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="G43" s="86"/>
       <c r="H43" s="85"/>
       <c r="I43" s="85"/>
       <c r="J43" s="85"/>
-      <c r="K43" s="84"/>
-      <c r="L43" s="127"/>
-      <c r="M43" s="86"/>
-      <c r="N43" s="86"/>
-      <c r="O43" s="86"/>
-      <c r="P43" s="86"/>
-      <c r="Q43" s="86"/>
+      <c r="K43" s="129"/>
+      <c r="L43" s="129"/>
+      <c r="M43" s="129"/>
+      <c r="N43" s="129"/>
+      <c r="O43" s="129"/>
+      <c r="P43" s="129"/>
+      <c r="Q43" s="129"/>
       <c r="R43" s="13">
         <f>SUM(G43:Q43)</f>
         <v>0</v>
@@ -3504,17 +3477,17 @@
     </row>
     <row r="44" spans="3:24" ht="67.5" customHeight="1">
       <c r="C44" s="60"/>
-      <c r="D44" s="6" t="s">
-        <v>29</v>
+      <c r="D44" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="E44" s="25"/>
       <c r="F44" s="45"/>
-      <c r="G44" s="91" t="str">
+      <c r="G44" s="89" t="str">
         <f>IF(G43=0, "", IF(MOD(G43, $F$43) = 0, G43/ $F$43, IF(INT(G43 / $F$43) = 0, MOD(G43, $F$43) &amp; " P", INT(G43 / $F$43) &amp; " + " &amp; MOD(G43, $F$43) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H44" s="90" t="str">
-        <f t="shared" ref="H44:Q44" si="8">IF(H43=0, "", IF(MOD(H43, $F$43) = 0, H43/ $F$43, IF(INT(H43 / $F$43) = 0, MOD(H43, $F$43) &amp; " P", INT(H43 / $F$43) &amp; " + " &amp; MOD(H43, $F$43) &amp; " P")))</f>
+        <f t="shared" ref="H44:L44" si="8">IF(H43=0, "", IF(MOD(H43, $F$43) = 0, H43/ $F$43, IF(INT(H43 / $F$43) = 0, MOD(H43, $F$43) &amp; " P", INT(H43 / $F$43) &amp; " + " &amp; MOD(H43, $F$43) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I44" s="90" t="str">
@@ -3525,110 +3498,110 @@
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="K44" s="91" t="str">
+      <c r="K44" s="89" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="L44" s="91" t="str">
+      <c r="L44" s="89" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="M44" s="91" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="N44" s="91" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O44" s="91" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="P44" s="91" t="str">
-        <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="Q44" s="91" t="str">
-        <f t="shared" si="8"/>
+      <c r="M44" s="89" t="str">
+        <f t="shared" ref="M44:Q44" si="9">IF(M43=0, "", IF(MOD(M43, $F$43) = 0, M43/ $F$43, IF(INT(M43 / $F$43) = 0, MOD(M43, $F$43) &amp; " P", INT(M43 / $F$43) &amp; " + " &amp; MOD(M43, $F$43) &amp; " P")))</f>
+        <v/>
+      </c>
+      <c r="N44" s="89" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="O44" s="89" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="P44" s="89" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="Q44" s="89" t="str">
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="R44" s="138">
         <f>G43+H43+I43+J43+K43+L43+O45</f>
-        <v>650</v>
+        <v>150</v>
       </c>
       <c r="S44" s="141">
         <f>O46</f>
-        <v>650</v>
+        <v>150</v>
       </c>
       <c r="X44" s="1"/>
     </row>
     <row r="45" spans="3:24" ht="67.5" customHeight="1">
       <c r="C45" s="60"/>
-      <c r="D45" s="7" t="s">
-        <v>33</v>
+      <c r="D45" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="E45" s="25"/>
       <c r="F45" s="45"/>
-      <c r="G45" s="112"/>
-      <c r="H45" s="95"/>
-      <c r="I45" s="96"/>
-      <c r="J45" s="97"/>
-      <c r="K45" s="99"/>
-      <c r="L45" s="112"/>
-      <c r="M45" s="100"/>
-      <c r="N45" s="100"/>
+      <c r="G45" s="130"/>
+      <c r="H45" s="131"/>
+      <c r="I45" s="131"/>
+      <c r="J45" s="131"/>
+      <c r="K45" s="132"/>
+      <c r="L45" s="132"/>
+      <c r="M45" s="132"/>
+      <c r="N45" s="132"/>
       <c r="O45" s="102">
-        <v>650</v>
-      </c>
-      <c r="P45" s="100"/>
-      <c r="Q45" s="113"/>
+        <v>150</v>
+      </c>
+      <c r="P45" s="132"/>
+      <c r="Q45" s="130"/>
       <c r="R45" s="139"/>
       <c r="S45" s="142"/>
       <c r="X45" s="1"/>
     </row>
     <row r="46" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C46" s="61"/>
-      <c r="D46" s="8" t="s">
+      <c r="D46" s="14" t="s">
         <v>8</v>
       </c>
       <c r="E46" s="26"/>
       <c r="F46" s="46"/>
-      <c r="G46" s="120"/>
-      <c r="H46" s="116"/>
-      <c r="I46" s="117"/>
-      <c r="J46" s="118"/>
-      <c r="K46" s="119"/>
-      <c r="L46" s="120"/>
-      <c r="M46" s="128"/>
-      <c r="N46" s="128"/>
-      <c r="O46" s="111">
+      <c r="G46" s="125"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="105"/>
+      <c r="J46" s="105"/>
+      <c r="K46" s="133"/>
+      <c r="L46" s="133"/>
+      <c r="M46" s="109"/>
+      <c r="N46" s="109"/>
+      <c r="O46" s="134">
         <f>SUM(O45-M43-N43-O43-P43-Q43)</f>
-        <v>650</v>
-      </c>
-      <c r="P46" s="128"/>
-      <c r="Q46" s="121"/>
+        <v>150</v>
+      </c>
+      <c r="P46" s="109"/>
+      <c r="Q46" s="126"/>
       <c r="R46" s="140"/>
-      <c r="S46" s="142"/>
+      <c r="S46" s="143"/>
       <c r="X46" s="1"/>
     </row>
     <row r="47" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C47" s="59">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D47" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="E47" s="24">
-        <v>43</v>
+        <v>55</v>
+      </c>
+      <c r="E47" s="27">
+        <v>79</v>
       </c>
       <c r="F47" s="44">
-        <v>20</v>
-      </c>
-      <c r="G47" s="86"/>
-      <c r="H47" s="85"/>
-      <c r="I47" s="85"/>
-      <c r="J47" s="85"/>
+        <v>15</v>
+      </c>
+      <c r="G47" s="129"/>
+      <c r="H47" s="135"/>
+      <c r="I47" s="135"/>
+      <c r="J47" s="135"/>
       <c r="K47" s="129"/>
       <c r="L47" s="129"/>
       <c r="M47" s="129"/>
@@ -3647,37 +3620,37 @@
     </row>
     <row r="48" spans="3:24" ht="67.5" customHeight="1">
       <c r="C48" s="60"/>
-      <c r="D48" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E48" s="25"/>
+      <c r="D48" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E48" s="28"/>
       <c r="F48" s="45"/>
       <c r="G48" s="89" t="str">
         <f>IF(G47=0, "", IF(MOD(G47, $F$47) = 0, G47/ $F$47, IF(INT(G47 / $F$47) = 0, MOD(G47, $F$47) &amp; " P", INT(G47 / $F$47) &amp; " + " &amp; MOD(G47, $F$47) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H48" s="90" t="str">
-        <f t="shared" ref="H48:L48" si="9">IF(H47=0, "", IF(MOD(H47, $F$47) = 0, H47/ $F$47, IF(INT(H47 / $F$47) = 0, MOD(H47, $F$47) &amp; " P", INT(H47 / $F$47) &amp; " + " &amp; MOD(H47, $F$47) &amp; " P")))</f>
+        <f t="shared" ref="H48:Q48" si="10">IF(H47=0, "", IF(MOD(H47, $F$47) = 0, H47/ $F$47, IF(INT(H47 / $F$47) = 0, MOD(H47, $F$47) &amp; " P", INT(H47 / $F$47) &amp; " + " &amp; MOD(H47, $F$47) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I48" s="90" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="J48" s="90" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="K48" s="89" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="L48" s="89" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="L48" si="11">IF(L47=0, "", IF(MOD(L47, $F$55) = 0, L47/ $F$55, IF(INT(L47 / $F$55) = 0, MOD(L47, $F$55) &amp; " P", INT(L47 / $F$55) &amp; " + " &amp; MOD(L47, $F$55) &amp; " P")))</f>
         <v/>
       </c>
       <c r="M48" s="89" t="str">
-        <f t="shared" ref="M48:Q48" si="10">IF(M47=0, "", IF(MOD(M47, $F$47) = 0, M47/ $F$47, IF(INT(M47 / $F$47) = 0, MOD(M47, $F$47) &amp; " P", INT(M47 / $F$47) &amp; " + " &amp; MOD(M47, $F$47) &amp; " P")))</f>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="N48" s="89" t="str">
@@ -3698,20 +3671,20 @@
       </c>
       <c r="R48" s="138">
         <f>G47+H47+I47+J47+K47+L47+O49</f>
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="S48" s="141">
         <f>O50</f>
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="X48" s="1"/>
     </row>
     <row r="49" spans="3:24" ht="67.5" customHeight="1">
       <c r="C49" s="60"/>
       <c r="D49" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E49" s="25"/>
+        <v>57</v>
+      </c>
+      <c r="E49" s="29"/>
       <c r="F49" s="45"/>
       <c r="G49" s="130"/>
       <c r="H49" s="131"/>
@@ -3721,8 +3694,8 @@
       <c r="L49" s="132"/>
       <c r="M49" s="132"/>
       <c r="N49" s="132"/>
-      <c r="O49" s="102">
-        <v>150</v>
+      <c r="O49" s="136">
+        <v>230</v>
       </c>
       <c r="P49" s="132"/>
       <c r="Q49" s="130"/>
@@ -3735,7 +3708,7 @@
       <c r="D50" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E50" s="26"/>
+      <c r="E50" s="30"/>
       <c r="F50" s="46"/>
       <c r="G50" s="125"/>
       <c r="H50" s="105"/>
@@ -3747,7 +3720,7 @@
       <c r="N50" s="109"/>
       <c r="O50" s="134">
         <f>SUM(O49-M47-N47-O47-P47-Q47)</f>
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="P50" s="109"/>
       <c r="Q50" s="126"/>
@@ -3757,16 +3730,16 @@
     </row>
     <row r="51" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C51" s="59">
-        <v>11</v>
-      </c>
-      <c r="D51" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="E51" s="27">
-        <v>79</v>
+        <v>12</v>
+      </c>
+      <c r="D51" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="E51" s="24">
+        <v>17</v>
       </c>
       <c r="F51" s="44">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="G51" s="129"/>
       <c r="H51" s="135"/>
@@ -3774,11 +3747,11 @@
       <c r="J51" s="135"/>
       <c r="K51" s="129"/>
       <c r="L51" s="129"/>
-      <c r="M51" s="129"/>
-      <c r="N51" s="129"/>
-      <c r="O51" s="129"/>
-      <c r="P51" s="129"/>
-      <c r="Q51" s="129"/>
+      <c r="M51" s="86"/>
+      <c r="N51" s="86"/>
+      <c r="O51" s="86"/>
+      <c r="P51" s="86"/>
+      <c r="Q51" s="86"/>
       <c r="R51" s="13">
         <f>SUM(G51:Q51)</f>
         <v>0</v>
@@ -3790,107 +3763,107 @@
     </row>
     <row r="52" spans="3:24" ht="67.5" customHeight="1">
       <c r="C52" s="60"/>
-      <c r="D52" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="E52" s="28"/>
+      <c r="D52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E52" s="25"/>
       <c r="F52" s="45"/>
-      <c r="G52" s="89" t="str">
-        <f>IF(G51=0, "", IF(MOD(G51, $F$51) = 0, G51/ $F$51, IF(INT(G51 / $F$51) = 0, MOD(G51, $F$51) &amp; " P", INT(G51 / $F$51) &amp; " + " &amp; MOD(G51, $F$51) &amp; " P")))</f>
+      <c r="G52" s="91" t="str">
+        <f>IF(G51=0, "", IF(MOD(G51, $F$51) = 0, G51 / $F$51, IF(INT(G51 / $F$51) = 0, MOD(G51, $F$51) &amp; " P", INT(G51 / $F$51) &amp; " + " &amp; MOD(G51, $F$51) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H52" s="90" t="str">
-        <f t="shared" ref="H52:Q52" si="11">IF(H51=0, "", IF(MOD(H51, $F$51) = 0, H51/ $F$51, IF(INT(H51 / $F$51) = 0, MOD(H51, $F$51) &amp; " P", INT(H51 / $F$51) &amp; " + " &amp; MOD(H51, $F$51) &amp; " P")))</f>
+        <f t="shared" ref="H52:L52" si="12">IF(H51=0, "", IF(MOD(H51, $F$51) = 0, H51 / $F$51, IF(INT(H51 / $F$51) = 0, MOD(H51, $F$51) &amp; " P", INT(H51 / $F$51) &amp; " + " &amp; MOD(H51, $F$51) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I52" s="90" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="J52" s="90" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="K52" s="89" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L52" s="89" t="str">
-        <f t="shared" ref="L52" si="12">IF(L51=0, "", IF(MOD(L51, $F$59) = 0, L51/ $F$59, IF(INT(L51 / $F$59) = 0, MOD(L51, $F$59) &amp; " P", INT(L51 / $F$59) &amp; " + " &amp; MOD(L51, $F$59) &amp; " P")))</f>
-        <v/>
-      </c>
-      <c r="M52" s="89" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="N52" s="89" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="O52" s="89" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="P52" s="89" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="Q52" s="89" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="K52" s="91" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="L52" s="91" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="M52" s="91" t="str">
+        <f>IF(M51=0, "", IF(MOD(M51, $F$51) = 0, M51 / $F$51, IF(INT(M51 / $F$51) = 0, MOD(M51, $F$51) &amp; " P", INT(M51 / $F$51) &amp; " + " &amp; MOD(M51, $F$51) &amp; " P")))</f>
+        <v/>
+      </c>
+      <c r="N52" s="91" t="str">
+        <f>IF(N51=0, "", IF(MOD(N51, $F$51) = 0, N51 / $F$51, IF(INT(N51 / $F$51) = 0, MOD(N51, $F$51) &amp; " P", INT(N51 / $F$51) &amp; " + " &amp; MOD(N51, $F$51) &amp; " P")))</f>
+        <v/>
+      </c>
+      <c r="O52" s="91" t="str">
+        <f>IF(O51=0, "", IF(MOD(O51, $F$51) = 0, O51 / $F$51, IF(INT(O51 / $F$51) = 0, MOD(O51, $F$51) &amp; " P", INT(O51 / $F$51) &amp; " + " &amp; MOD(O51, $F$51) &amp; " P")))</f>
+        <v/>
+      </c>
+      <c r="P52" s="91" t="str">
+        <f>IF(P51=0, "", IF(MOD(P51, $F$51) = 0, P51 / $F$51, IF(INT(P51 / $F$51) = 0, MOD(P51, $F$51) &amp; " P", INT(P51 / $F$51) &amp; " + " &amp; MOD(P51, $F$51) &amp; " P")))</f>
+        <v/>
+      </c>
+      <c r="Q52" s="91" t="str">
+        <f>IF(Q51=0, "", IF(MOD(Q51, $F$51) = 0, Q51 / $F$51, IF(INT(Q51 / $F$51) = 0, MOD(Q51, $F$51) &amp; " P", INT(Q51 / $F$51) &amp; " + " &amp; MOD(Q51, $F$51) &amp; " P")))</f>
         <v/>
       </c>
       <c r="R52" s="138">
         <f>G51+H51+I51+J51+K51+L51+O53</f>
-        <v>230</v>
+        <v>60</v>
       </c>
       <c r="S52" s="141">
-        <f>O54</f>
-        <v>230</v>
+        <f>SUM(O54)</f>
+        <v>60</v>
       </c>
       <c r="X52" s="1"/>
     </row>
     <row r="53" spans="3:24" ht="67.5" customHeight="1">
       <c r="C53" s="60"/>
-      <c r="D53" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E53" s="29"/>
+      <c r="D53" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E53" s="25"/>
       <c r="F53" s="45"/>
-      <c r="G53" s="130"/>
-      <c r="H53" s="131"/>
-      <c r="I53" s="131"/>
-      <c r="J53" s="131"/>
-      <c r="K53" s="132"/>
-      <c r="L53" s="132"/>
-      <c r="M53" s="132"/>
-      <c r="N53" s="132"/>
-      <c r="O53" s="136">
-        <v>230</v>
-      </c>
-      <c r="P53" s="132"/>
-      <c r="Q53" s="130"/>
+      <c r="G53" s="112"/>
+      <c r="H53" s="95"/>
+      <c r="I53" s="96"/>
+      <c r="J53" s="97"/>
+      <c r="K53" s="99"/>
+      <c r="L53" s="112"/>
+      <c r="M53" s="100"/>
+      <c r="N53" s="100"/>
+      <c r="O53" s="102">
+        <v>60</v>
+      </c>
+      <c r="P53" s="100"/>
+      <c r="Q53" s="113"/>
       <c r="R53" s="139"/>
       <c r="S53" s="142"/>
       <c r="X53" s="1"/>
     </row>
     <row r="54" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C54" s="61"/>
-      <c r="D54" s="14" t="s">
+      <c r="D54" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E54" s="30"/>
+      <c r="E54" s="26"/>
       <c r="F54" s="46"/>
       <c r="G54" s="125"/>
-      <c r="H54" s="105"/>
+      <c r="H54" s="104"/>
       <c r="I54" s="105"/>
-      <c r="J54" s="105"/>
-      <c r="K54" s="133"/>
-      <c r="L54" s="133"/>
+      <c r="J54" s="106"/>
+      <c r="K54" s="108"/>
+      <c r="L54" s="125"/>
       <c r="M54" s="109"/>
       <c r="N54" s="109"/>
-      <c r="O54" s="134">
+      <c r="O54" s="111">
         <f>SUM(O53-M51-N51-O51-P51-Q51)</f>
-        <v>230</v>
+        <v>60</v>
       </c>
       <c r="P54" s="109"/>
       <c r="Q54" s="126"/>
@@ -3900,16 +3873,16 @@
     </row>
     <row r="55" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C55" s="59">
-        <v>12</v>
-      </c>
-      <c r="D55" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="E55" s="24">
-        <v>17</v>
+        <v>13</v>
+      </c>
+      <c r="D55" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E55" s="27">
+        <v>59.3</v>
       </c>
       <c r="F55" s="44">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G55" s="129"/>
       <c r="H55" s="135"/>
@@ -3917,11 +3890,11 @@
       <c r="J55" s="135"/>
       <c r="K55" s="129"/>
       <c r="L55" s="129"/>
-      <c r="M55" s="86"/>
-      <c r="N55" s="86"/>
-      <c r="O55" s="86"/>
-      <c r="P55" s="86"/>
-      <c r="Q55" s="86"/>
+      <c r="M55" s="129"/>
+      <c r="N55" s="129"/>
+      <c r="O55" s="129"/>
+      <c r="P55" s="129"/>
+      <c r="Q55" s="129"/>
       <c r="R55" s="13">
         <f>SUM(G55:Q55)</f>
         <v>0</v>
@@ -3933,17 +3906,17 @@
     </row>
     <row r="56" spans="3:24" ht="67.5" customHeight="1">
       <c r="C56" s="60"/>
-      <c r="D56" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E56" s="25"/>
+      <c r="D56" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="E56" s="29"/>
       <c r="F56" s="45"/>
-      <c r="G56" s="91" t="str">
-        <f>IF(G55=0, "", IF(MOD(G55, $F$55) = 0, G55 / $F$55, IF(INT(G55 / $F$55) = 0, MOD(G55, $F$55) &amp; " P", INT(G55 / $F$55) &amp; " + " &amp; MOD(G55, $F$55) &amp; " P")))</f>
+      <c r="G56" s="89" t="str">
+        <f>IF(G55=0, "", IF(MOD(G55, $F$55) = 0, G55/ $F$55, IF(INT(G55 / $F$55) = 0, MOD(G55, $F$55) &amp; " P", INT(G55 / $F$55) &amp; " + " &amp; MOD(G55, $F$55) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H56" s="90" t="str">
-        <f t="shared" ref="H56:L56" si="13">IF(H55=0, "", IF(MOD(H55, $F$55) = 0, H55 / $F$55, IF(INT(H55 / $F$55) = 0, MOD(H55, $F$55) &amp; " P", INT(H55 / $F$55) &amp; " + " &amp; MOD(H55, $F$55) &amp; " P")))</f>
+        <f t="shared" ref="H56:Q56" si="13">IF(H55=0, "", IF(MOD(H55, $F$55) = 0, H55/ $F$55, IF(INT(H55 / $F$55) = 0, MOD(H55, $F$55) &amp; " P", INT(H55 / $F$55) &amp; " + " &amp; MOD(H55, $F$55) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I56" s="90" t="str">
@@ -3954,86 +3927,86 @@
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="K56" s="91" t="str">
+      <c r="K56" s="89" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="L56" s="91" t="str">
+      <c r="L56" s="89" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="M56" s="91" t="str">
-        <f>IF(M55=0, "", IF(MOD(M55, $F$55) = 0, M55 / $F$55, IF(INT(M55 / $F$55) = 0, MOD(M55, $F$55) &amp; " P", INT(M55 / $F$55) &amp; " + " &amp; MOD(M55, $F$55) &amp; " P")))</f>
-        <v/>
-      </c>
-      <c r="N56" s="91" t="str">
-        <f>IF(N55=0, "", IF(MOD(N55, $F$55) = 0, N55 / $F$55, IF(INT(N55 / $F$55) = 0, MOD(N55, $F$55) &amp; " P", INT(N55 / $F$55) &amp; " + " &amp; MOD(N55, $F$55) &amp; " P")))</f>
-        <v/>
-      </c>
-      <c r="O56" s="91" t="str">
-        <f>IF(O55=0, "", IF(MOD(O55, $F$55) = 0, O55 / $F$55, IF(INT(O55 / $F$55) = 0, MOD(O55, $F$55) &amp; " P", INT(O55 / $F$55) &amp; " + " &amp; MOD(O55, $F$55) &amp; " P")))</f>
-        <v/>
-      </c>
-      <c r="P56" s="91" t="str">
-        <f>IF(P55=0, "", IF(MOD(P55, $F$55) = 0, P55 / $F$55, IF(INT(P55 / $F$55) = 0, MOD(P55, $F$55) &amp; " P", INT(P55 / $F$55) &amp; " + " &amp; MOD(P55, $F$55) &amp; " P")))</f>
-        <v/>
-      </c>
-      <c r="Q56" s="91" t="str">
-        <f>IF(Q55=0, "", IF(MOD(Q55, $F$55) = 0, Q55 / $F$55, IF(INT(Q55 / $F$55) = 0, MOD(Q55, $F$55) &amp; " P", INT(Q55 / $F$55) &amp; " + " &amp; MOD(Q55, $F$55) &amp; " P")))</f>
+      <c r="M56" s="89" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="N56" s="89" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="O56" s="89" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="P56" s="89" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="Q56" s="89" t="str">
+        <f t="shared" si="13"/>
         <v/>
       </c>
       <c r="R56" s="138">
         <f>G55+H55+I55+J55+K55+L55+O57</f>
-        <v>60</v>
+        <v>270</v>
       </c>
       <c r="S56" s="141">
-        <f>SUM(O58)</f>
-        <v>60</v>
+        <f>O58</f>
+        <v>270</v>
       </c>
       <c r="X56" s="1"/>
     </row>
     <row r="57" spans="3:24" ht="67.5" customHeight="1">
       <c r="C57" s="60"/>
-      <c r="D57" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E57" s="25"/>
+      <c r="D57" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="E57" s="29"/>
       <c r="F57" s="45"/>
-      <c r="G57" s="112"/>
-      <c r="H57" s="95"/>
-      <c r="I57" s="96"/>
-      <c r="J57" s="97"/>
-      <c r="K57" s="99"/>
-      <c r="L57" s="112"/>
-      <c r="M57" s="100"/>
-      <c r="N57" s="100"/>
+      <c r="G57" s="130"/>
+      <c r="H57" s="131"/>
+      <c r="I57" s="131"/>
+      <c r="J57" s="131"/>
+      <c r="K57" s="132"/>
+      <c r="L57" s="132"/>
+      <c r="M57" s="132"/>
+      <c r="N57" s="132"/>
       <c r="O57" s="102">
-        <v>60</v>
-      </c>
-      <c r="P57" s="100"/>
-      <c r="Q57" s="113"/>
+        <v>270</v>
+      </c>
+      <c r="P57" s="132"/>
+      <c r="Q57" s="130"/>
       <c r="R57" s="139"/>
       <c r="S57" s="142"/>
       <c r="X57" s="1"/>
     </row>
     <row r="58" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C58" s="61"/>
-      <c r="D58" s="8" t="s">
+      <c r="D58" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E58" s="26"/>
+      <c r="E58" s="30"/>
       <c r="F58" s="46"/>
       <c r="G58" s="125"/>
-      <c r="H58" s="104"/>
+      <c r="H58" s="105"/>
       <c r="I58" s="105"/>
-      <c r="J58" s="106"/>
-      <c r="K58" s="108"/>
-      <c r="L58" s="125"/>
+      <c r="J58" s="105"/>
+      <c r="K58" s="133"/>
+      <c r="L58" s="133"/>
       <c r="M58" s="109"/>
       <c r="N58" s="109"/>
-      <c r="O58" s="111">
+      <c r="O58" s="134">
         <f>SUM(O57-M55-N55-O55-P55-Q55)</f>
-        <v>60</v>
+        <v>270</v>
       </c>
       <c r="P58" s="109"/>
       <c r="Q58" s="126"/>
@@ -4043,13 +4016,13 @@
     </row>
     <row r="59" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C59" s="59">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D59" s="21" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="E59" s="27">
-        <v>59.3</v>
+        <v>66.5</v>
       </c>
       <c r="F59" s="44">
         <v>15</v>
@@ -4077,7 +4050,7 @@
     <row r="60" spans="3:24" ht="67.5" customHeight="1">
       <c r="C60" s="60"/>
       <c r="D60" s="16" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E60" s="29"/>
       <c r="F60" s="45"/>
@@ -4127,18 +4100,18 @@
       </c>
       <c r="R60" s="138">
         <f>G59+H59+I59+J59+K59+L59+O61</f>
-        <v>270</v>
+        <v>120</v>
       </c>
       <c r="S60" s="141">
         <f>O62</f>
-        <v>270</v>
+        <v>120</v>
       </c>
       <c r="X60" s="1"/>
     </row>
     <row r="61" spans="3:24" ht="67.5" customHeight="1">
       <c r="C61" s="60"/>
       <c r="D61" s="11" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E61" s="29"/>
       <c r="F61" s="45"/>
@@ -4151,7 +4124,7 @@
       <c r="M61" s="132"/>
       <c r="N61" s="132"/>
       <c r="O61" s="102">
-        <v>270</v>
+        <v>120</v>
       </c>
       <c r="P61" s="132"/>
       <c r="Q61" s="130"/>
@@ -4176,7 +4149,7 @@
       <c r="N62" s="109"/>
       <c r="O62" s="134">
         <f>SUM(O61-M59-N59-O59-P59-Q59)</f>
-        <v>270</v>
+        <v>120</v>
       </c>
       <c r="P62" s="109"/>
       <c r="Q62" s="126"/>
@@ -4186,16 +4159,16 @@
     </row>
     <row r="63" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C63" s="59">
-        <v>14</v>
-      </c>
-      <c r="D63" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="E63" s="27">
-        <v>66.5</v>
-      </c>
-      <c r="F63" s="44">
         <v>15</v>
+      </c>
+      <c r="D63" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E63" s="24">
+        <v>34</v>
+      </c>
+      <c r="F63" s="47">
+        <v>27</v>
       </c>
       <c r="G63" s="129"/>
       <c r="H63" s="135"/>
@@ -4219,17 +4192,17 @@
     </row>
     <row r="64" spans="3:24" ht="67.5" customHeight="1">
       <c r="C64" s="60"/>
-      <c r="D64" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="E64" s="29"/>
-      <c r="F64" s="45"/>
+      <c r="D64" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E64" s="25"/>
+      <c r="F64" s="48"/>
       <c r="G64" s="89" t="str">
         <f>IF(G63=0, "", IF(MOD(G63, $F$63) = 0, G63/ $F$63, IF(INT(G63 / $F$63) = 0, MOD(G63, $F$63) &amp; " P", INT(G63 / $F$63) &amp; " + " &amp; MOD(G63, $F$63) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H64" s="90" t="str">
-        <f t="shared" ref="H64:Q64" si="15">IF(H63=0, "", IF(MOD(H63, $F$63) = 0, H63/ $F$63, IF(INT(H63 / $F$63) = 0, MOD(H63, $F$63) &amp; " P", INT(H63 / $F$63) &amp; " + " &amp; MOD(H63, $F$63) &amp; " P")))</f>
+        <f t="shared" ref="H64:M64" si="15">IF(H63=0, "", IF(MOD(H63, $F$63) = 0, H63/ $F$63, IF(INT(H63 / $F$63) = 0, MOD(H63, $F$63) &amp; " P", INT(H63 / $F$63) &amp; " + " &amp; MOD(H63, $F$63) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I64" s="90" t="str">
@@ -4253,38 +4226,38 @@
         <v/>
       </c>
       <c r="N64" s="89" t="str">
-        <f t="shared" si="15"/>
+        <f>IF(N63=0, "", IF(MOD(N63, $F$63) = 0, N63/ $F$63, IF(INT(N63 / $F$63) = 0, MOD(N63, $F$63) &amp; " P", INT(N63 / $F$63) &amp; " + " &amp; MOD(N63, $F$63) &amp; " P")))</f>
         <v/>
       </c>
       <c r="O64" s="89" t="str">
-        <f t="shared" si="15"/>
+        <f>IF(O63=0, "", IF(MOD(O63, $F$63) = 0, O63/ $F$63, IF(INT(O63 / $F$63) = 0, MOD(O63, $F$63) &amp; " P", INT(O63 / $F$63) &amp; " + " &amp; MOD(O63, $F$63) &amp; " P")))</f>
         <v/>
       </c>
       <c r="P64" s="89" t="str">
-        <f t="shared" si="15"/>
+        <f>IF(P63=0, "", IF(MOD(P63, $F$63) = 0, P63/ $F$63, IF(INT(P63 / $F$63) = 0, MOD(P63, $F$63) &amp; " P", INT(P63 / $F$63) &amp; " + " &amp; MOD(P63, $F$63) &amp; " P")))</f>
         <v/>
       </c>
       <c r="Q64" s="89" t="str">
-        <f t="shared" si="15"/>
+        <f>IF(Q63=0, "", IF(MOD(Q63, $F$63) = 0, Q63/ $F$63, IF(INT(Q63 / $F$63) = 0, MOD(Q63, $F$63) &amp; " P", INT(Q63 / $F$63) &amp; " + " &amp; MOD(Q63, $F$63) &amp; " P")))</f>
         <v/>
       </c>
       <c r="R64" s="138">
         <f>G63+H63+I63+J63+K63+L63+O65</f>
-        <v>120</v>
+        <v>320</v>
       </c>
       <c r="S64" s="141">
         <f>O66</f>
-        <v>120</v>
+        <v>320</v>
       </c>
       <c r="X64" s="1"/>
     </row>
     <row r="65" spans="3:24" ht="67.5" customHeight="1">
       <c r="C65" s="60"/>
-      <c r="D65" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E65" s="29"/>
-      <c r="F65" s="45"/>
+      <c r="D65" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E65" s="25"/>
+      <c r="F65" s="48"/>
       <c r="G65" s="130"/>
       <c r="H65" s="131"/>
       <c r="I65" s="131"/>
@@ -4293,8 +4266,8 @@
       <c r="L65" s="132"/>
       <c r="M65" s="132"/>
       <c r="N65" s="132"/>
-      <c r="O65" s="102">
-        <v>120</v>
+      <c r="O65" s="136">
+        <v>320</v>
       </c>
       <c r="P65" s="132"/>
       <c r="Q65" s="130"/>
@@ -4307,8 +4280,8 @@
       <c r="D66" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E66" s="30"/>
-      <c r="F66" s="46"/>
+      <c r="E66" s="26"/>
+      <c r="F66" s="49"/>
       <c r="G66" s="125"/>
       <c r="H66" s="105"/>
       <c r="I66" s="105"/>
@@ -4319,7 +4292,7 @@
       <c r="N66" s="109"/>
       <c r="O66" s="134">
         <f>SUM(O65-M63-N63-O63-P63-Q63)</f>
-        <v>120</v>
+        <v>320</v>
       </c>
       <c r="P66" s="109"/>
       <c r="Q66" s="126"/>
@@ -4329,16 +4302,16 @@
     </row>
     <row r="67" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C67" s="59">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D67" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="E67" s="24">
-        <v>34</v>
+        <v>22</v>
+      </c>
+      <c r="E67" s="34">
+        <v>42</v>
       </c>
       <c r="F67" s="47">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="G67" s="129"/>
       <c r="H67" s="135"/>
@@ -4346,11 +4319,11 @@
       <c r="J67" s="135"/>
       <c r="K67" s="129"/>
       <c r="L67" s="129"/>
-      <c r="M67" s="129"/>
-      <c r="N67" s="129"/>
-      <c r="O67" s="129"/>
-      <c r="P67" s="129"/>
-      <c r="Q67" s="129"/>
+      <c r="M67" s="86"/>
+      <c r="N67" s="86"/>
+      <c r="O67" s="86"/>
+      <c r="P67" s="86"/>
+      <c r="Q67" s="86"/>
       <c r="R67" s="13">
         <f>SUM(G67:Q67)</f>
         <v>0</v>
@@ -4363,16 +4336,16 @@
     <row r="68" spans="3:24" ht="67.5" customHeight="1">
       <c r="C68" s="60"/>
       <c r="D68" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E68" s="25"/>
+        <v>27</v>
+      </c>
+      <c r="E68" s="35"/>
       <c r="F68" s="48"/>
       <c r="G68" s="89" t="str">
         <f>IF(G67=0, "", IF(MOD(G67, $F$67) = 0, G67/ $F$67, IF(INT(G67 / $F$67) = 0, MOD(G67, $F$67) &amp; " P", INT(G67 / $F$67) &amp; " + " &amp; MOD(G67, $F$67) &amp; " P")))</f>
         <v/>
       </c>
       <c r="H68" s="90" t="str">
-        <f t="shared" ref="H68:M68" si="16">IF(H67=0, "", IF(MOD(H67, $F$67) = 0, H67/ $F$67, IF(INT(H67 / $F$67) = 0, MOD(H67, $F$67) &amp; " P", INT(H67 / $F$67) &amp; " + " &amp; MOD(H67, $F$67) &amp; " P")))</f>
+        <f t="shared" ref="H68:Q68" si="16">IF(H67=0, "", IF(MOD(H67, $F$67) = 0, H67/ $F$67, IF(INT(H67 / $F$67) = 0, MOD(H67, $F$67) &amp; " P", INT(H67 / $F$67) &amp; " + " &amp; MOD(H67, $F$67) &amp; " P")))</f>
         <v/>
       </c>
       <c r="I68" s="90" t="str">
@@ -4396,37 +4369,37 @@
         <v/>
       </c>
       <c r="N68" s="89" t="str">
-        <f>IF(N67=0, "", IF(MOD(N67, $F$67) = 0, N67/ $F$67, IF(INT(N67 / $F$67) = 0, MOD(N67, $F$67) &amp; " P", INT(N67 / $F$67) &amp; " + " &amp; MOD(N67, $F$67) &amp; " P")))</f>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="O68" s="89" t="str">
-        <f>IF(O67=0, "", IF(MOD(O67, $F$67) = 0, O67/ $F$67, IF(INT(O67 / $F$67) = 0, MOD(O67, $F$67) &amp; " P", INT(O67 / $F$67) &amp; " + " &amp; MOD(O67, $F$67) &amp; " P")))</f>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="P68" s="89" t="str">
-        <f>IF(P67=0, "", IF(MOD(P67, $F$67) = 0, P67/ $F$67, IF(INT(P67 / $F$67) = 0, MOD(P67, $F$67) &amp; " P", INT(P67 / $F$67) &amp; " + " &amp; MOD(P67, $F$67) &amp; " P")))</f>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="Q68" s="89" t="str">
-        <f>IF(Q67=0, "", IF(MOD(Q67, $F$67) = 0, Q67/ $F$67, IF(INT(Q67 / $F$67) = 0, MOD(Q67, $F$67) &amp; " P", INT(Q67 / $F$67) &amp; " + " &amp; MOD(Q67, $F$67) &amp; " P")))</f>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="R68" s="138">
         <f>G67+H67+I67+J67+K67+L67+O69</f>
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="S68" s="141">
         <f>O70</f>
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="X68" s="1"/>
     </row>
     <row r="69" spans="3:24" ht="67.5" customHeight="1">
       <c r="C69" s="60"/>
       <c r="D69" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="E69" s="25"/>
+        <v>31</v>
+      </c>
+      <c r="E69" s="35"/>
       <c r="F69" s="48"/>
       <c r="G69" s="130"/>
       <c r="H69" s="131"/>
@@ -4437,7 +4410,7 @@
       <c r="M69" s="132"/>
       <c r="N69" s="132"/>
       <c r="O69" s="136">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="P69" s="132"/>
       <c r="Q69" s="130"/>
@@ -4462,7 +4435,7 @@
       <c r="N70" s="109"/>
       <c r="O70" s="134">
         <f>SUM(O69-M67-N67-O67-P67-Q67)</f>
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="P70" s="109"/>
       <c r="Q70" s="126"/>
@@ -4472,16 +4445,16 @@
     </row>
     <row r="71" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
       <c r="C71" s="59">
-        <v>16</v>
-      </c>
-      <c r="D71" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="E71" s="34">
-        <v>42</v>
-      </c>
-      <c r="F71" s="47">
-        <v>20</v>
+        <v>17</v>
+      </c>
+      <c r="D71" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="E71" s="31">
+        <v>90</v>
+      </c>
+      <c r="F71" s="44">
+        <v>32</v>
       </c>
       <c r="G71" s="129"/>
       <c r="H71" s="135"/>
@@ -4506,10 +4479,10 @@
     <row r="72" spans="3:24" ht="67.5" customHeight="1">
       <c r="C72" s="60"/>
       <c r="D72" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E72" s="35"/>
-      <c r="F72" s="48"/>
+        <v>28</v>
+      </c>
+      <c r="E72" s="32"/>
+      <c r="F72" s="45"/>
       <c r="G72" s="89" t="str">
         <f>IF(G71=0, "", IF(MOD(G71, $F$71) = 0, G71/ $F$71, IF(INT(G71 / $F$71) = 0, MOD(G71, $F$71) &amp; " P", INT(G71 / $F$71) &amp; " + " &amp; MOD(G71, $F$71) &amp; " P")))</f>
         <v/>
@@ -4556,21 +4529,21 @@
       </c>
       <c r="R72" s="138">
         <f>G71+H71+I71+J71+K71+L71+O73</f>
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="S72" s="141">
         <f>O74</f>
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="X72" s="1"/>
     </row>
     <row r="73" spans="3:24" ht="67.5" customHeight="1">
       <c r="C73" s="60"/>
       <c r="D73" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E73" s="35"/>
-      <c r="F73" s="48"/>
+        <v>30</v>
+      </c>
+      <c r="E73" s="32"/>
+      <c r="F73" s="45"/>
       <c r="G73" s="130"/>
       <c r="H73" s="131"/>
       <c r="I73" s="131"/>
@@ -4580,7 +4553,7 @@
       <c r="M73" s="132"/>
       <c r="N73" s="132"/>
       <c r="O73" s="136">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="P73" s="132"/>
       <c r="Q73" s="130"/>
@@ -4593,8 +4566,8 @@
       <c r="D74" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E74" s="26"/>
-      <c r="F74" s="49"/>
+      <c r="E74" s="33"/>
+      <c r="F74" s="46"/>
       <c r="G74" s="125"/>
       <c r="H74" s="105"/>
       <c r="I74" s="105"/>
@@ -4605,7 +4578,7 @@
       <c r="N74" s="109"/>
       <c r="O74" s="134">
         <f>SUM(O73-M71-N71-O71-P71-Q71)</f>
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="P74" s="109"/>
       <c r="Q74" s="126"/>
@@ -4614,17 +4587,17 @@
       <c r="X74" s="1"/>
     </row>
     <row r="75" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C75" s="59">
-        <v>17</v>
-      </c>
-      <c r="D75" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="E75" s="31">
-        <v>90</v>
-      </c>
-      <c r="F75" s="44">
-        <v>32</v>
+      <c r="C75" s="68">
+        <v>18</v>
+      </c>
+      <c r="D75" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="E75" s="27">
+        <v>31.16</v>
+      </c>
+      <c r="F75" s="71">
+        <v>15</v>
       </c>
       <c r="G75" s="129"/>
       <c r="H75" s="135"/>
@@ -4647,12 +4620,12 @@
       <c r="X75" s="1"/>
     </row>
     <row r="76" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C76" s="60"/>
-      <c r="D76" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E76" s="32"/>
-      <c r="F76" s="45"/>
+      <c r="C76" s="69"/>
+      <c r="D76" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E76" s="29"/>
+      <c r="F76" s="72"/>
       <c r="G76" s="89" t="str">
         <f>IF(G75=0, "", IF(MOD(G75, $F$75) = 0, G75/ $F$75, IF(INT(G75 / $F$75) = 0, MOD(G75, $F$75) &amp; " P", INT(G75 / $F$75) &amp; " + " &amp; MOD(G75, $F$75) &amp; " P")))</f>
         <v/>
@@ -4708,12 +4681,12 @@
       <c r="X76" s="1"/>
     </row>
     <row r="77" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C77" s="60"/>
-      <c r="D77" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E77" s="32"/>
-      <c r="F77" s="45"/>
+      <c r="C77" s="69"/>
+      <c r="D77" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E77" s="29"/>
+      <c r="F77" s="72"/>
       <c r="G77" s="130"/>
       <c r="H77" s="131"/>
       <c r="I77" s="131"/>
@@ -4732,12 +4705,12 @@
       <c r="X77" s="1"/>
     </row>
     <row r="78" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C78" s="61"/>
+      <c r="C78" s="70"/>
       <c r="D78" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E78" s="33"/>
-      <c r="F78" s="46"/>
+      <c r="E78" s="30"/>
+      <c r="F78" s="73"/>
       <c r="G78" s="125"/>
       <c r="H78" s="105"/>
       <c r="I78" s="105"/>
@@ -4757,17 +4730,17 @@
       <c r="X78" s="1"/>
     </row>
     <row r="79" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C79" s="68">
-        <v>18</v>
-      </c>
-      <c r="D79" s="21" t="s">
-        <v>35</v>
+      <c r="C79" s="81">
+        <v>19</v>
+      </c>
+      <c r="D79" s="137" t="s">
+        <v>77</v>
       </c>
       <c r="E79" s="27">
-        <v>31.16</v>
-      </c>
-      <c r="F79" s="71">
-        <v>15</v>
+        <v>62.31</v>
+      </c>
+      <c r="F79" s="78">
+        <v>8</v>
       </c>
       <c r="G79" s="129"/>
       <c r="H79" s="135"/>
@@ -4790,12 +4763,12 @@
       <c r="X79" s="1"/>
     </row>
     <row r="80" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C80" s="69"/>
+      <c r="C80" s="82"/>
       <c r="D80" s="16" t="s">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="E80" s="29"/>
-      <c r="F80" s="72"/>
+      <c r="F80" s="79"/>
       <c r="G80" s="89" t="str">
         <f>IF(G79=0, "", IF(MOD(G79, $F$79) = 0, G79/ $F$79, IF(INT(G79 / $F$79) = 0, MOD(G79, $F$79) &amp; " P", INT(G79 / $F$79) &amp; " + " &amp; MOD(G79, $F$79) &amp; " P")))</f>
         <v/>
@@ -4851,12 +4824,12 @@
       <c r="X80" s="1"/>
     </row>
     <row r="81" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C81" s="69"/>
+      <c r="C81" s="82"/>
       <c r="D81" s="11" t="s">
-        <v>37</v>
+        <v>79</v>
       </c>
       <c r="E81" s="29"/>
-      <c r="F81" s="72"/>
+      <c r="F81" s="79"/>
       <c r="G81" s="130"/>
       <c r="H81" s="131"/>
       <c r="I81" s="131"/>
@@ -4875,12 +4848,12 @@
       <c r="X81" s="1"/>
     </row>
     <row r="82" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C82" s="70"/>
+      <c r="C82" s="83"/>
       <c r="D82" s="14" t="s">
         <v>8</v>
       </c>
       <c r="E82" s="30"/>
-      <c r="F82" s="73"/>
+      <c r="F82" s="80"/>
       <c r="G82" s="125"/>
       <c r="H82" s="105"/>
       <c r="I82" s="105"/>
@@ -4899,149 +4872,10 @@
       <c r="S82" s="143"/>
       <c r="X82" s="1"/>
     </row>
-    <row r="83" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C83" s="81">
-        <v>19</v>
-      </c>
-      <c r="D83" s="137" t="s">
-        <v>80</v>
-      </c>
-      <c r="E83" s="27">
-        <v>62.31</v>
-      </c>
-      <c r="F83" s="78">
-        <v>8</v>
-      </c>
-      <c r="G83" s="129"/>
-      <c r="H83" s="135"/>
-      <c r="I83" s="135"/>
-      <c r="J83" s="135"/>
-      <c r="K83" s="129"/>
-      <c r="L83" s="129"/>
-      <c r="M83" s="86"/>
-      <c r="N83" s="86"/>
-      <c r="O83" s="86"/>
-      <c r="P83" s="86"/>
-      <c r="Q83" s="86"/>
-      <c r="R83" s="13">
-        <f>SUM(G83:Q83)</f>
-        <v>0</v>
-      </c>
-      <c r="S83" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="X83" s="1"/>
-    </row>
-    <row r="84" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C84" s="82"/>
-      <c r="D84" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="E84" s="29"/>
-      <c r="F84" s="79"/>
-      <c r="G84" s="89" t="str">
-        <f>IF(G83=0, "", IF(MOD(G83, $F$83) = 0, G83/ $F$83, IF(INT(G83 / $F$83) = 0, MOD(G83, $F$83) &amp; " P", INT(G83 / $F$83) &amp; " + " &amp; MOD(G83, $F$83) &amp; " P")))</f>
-        <v/>
-      </c>
-      <c r="H84" s="90" t="str">
-        <f t="shared" ref="H84:Q84" si="20">IF(H83=0, "", IF(MOD(H83, $F$83) = 0, H83/ $F$83, IF(INT(H83 / $F$83) = 0, MOD(H83, $F$83) &amp; " P", INT(H83 / $F$83) &amp; " + " &amp; MOD(H83, $F$83) &amp; " P")))</f>
-        <v/>
-      </c>
-      <c r="I84" s="90" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="J84" s="90" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="K84" s="89" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="L84" s="89" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="M84" s="89" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="N84" s="89" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="O84" s="89" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="P84" s="89" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="Q84" s="89" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="R84" s="138">
-        <f>G83+H83+I83+J83+K83+L83+O85</f>
-        <v>100</v>
-      </c>
-      <c r="S84" s="141">
-        <f>O86</f>
-        <v>100</v>
-      </c>
-      <c r="X84" s="1"/>
-    </row>
-    <row r="85" spans="3:24" ht="67.5" customHeight="1">
-      <c r="C85" s="82"/>
-      <c r="D85" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="E85" s="29"/>
-      <c r="F85" s="79"/>
-      <c r="G85" s="130"/>
-      <c r="H85" s="131"/>
-      <c r="I85" s="131"/>
-      <c r="J85" s="131"/>
-      <c r="K85" s="132"/>
-      <c r="L85" s="132"/>
-      <c r="M85" s="132"/>
-      <c r="N85" s="132"/>
-      <c r="O85" s="136">
-        <v>100</v>
-      </c>
-      <c r="P85" s="132"/>
-      <c r="Q85" s="130"/>
-      <c r="R85" s="139"/>
-      <c r="S85" s="142"/>
-      <c r="X85" s="1"/>
-    </row>
-    <row r="86" spans="3:24" ht="67.5" customHeight="1" thickBot="1">
-      <c r="C86" s="83"/>
-      <c r="D86" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="E86" s="30"/>
-      <c r="F86" s="80"/>
-      <c r="G86" s="125"/>
-      <c r="H86" s="105"/>
-      <c r="I86" s="105"/>
-      <c r="J86" s="105"/>
-      <c r="K86" s="133"/>
-      <c r="L86" s="133"/>
-      <c r="M86" s="109"/>
-      <c r="N86" s="109"/>
-      <c r="O86" s="134">
-        <f>SUM(O85-M83-N83-O83-P83-Q83)</f>
-        <v>100</v>
-      </c>
-      <c r="P86" s="109"/>
-      <c r="Q86" s="126"/>
-      <c r="R86" s="140"/>
-      <c r="S86" s="143"/>
-      <c r="X86" s="1"/>
-    </row>
+    <row r="83" spans="3:24" ht="73.5" customHeight="1"/>
+    <row r="84" spans="3:24" ht="73.5" customHeight="1"/>
+    <row r="85" spans="3:24" ht="73.5" customHeight="1"/>
+    <row r="86" spans="3:24" ht="73.5" customHeight="1"/>
     <row r="87" spans="3:24" ht="73.5" customHeight="1"/>
     <row r="88" spans="3:24" ht="73.5" customHeight="1"/>
     <row r="89" spans="3:24" ht="73.5" customHeight="1"/>
@@ -5060,41 +4894,40 @@
     <row r="102" ht="73.5" customHeight="1"/>
     <row r="103" ht="73.5" customHeight="1"/>
     <row r="104" ht="73.5" customHeight="1"/>
-    <row r="105" ht="73.5" customHeight="1"/>
-    <row r="106" ht="73.5" customHeight="1"/>
-    <row r="107" ht="73.5" customHeight="1"/>
-    <row r="108" ht="73.5" customHeight="1"/>
   </sheetData>
-  <mergeCells count="78">
-    <mergeCell ref="R84:R86"/>
-    <mergeCell ref="S84:S86"/>
+  <mergeCells count="73">
+    <mergeCell ref="R56:R58"/>
+    <mergeCell ref="S56:S58"/>
+    <mergeCell ref="S52:S54"/>
+    <mergeCell ref="R52:R54"/>
+    <mergeCell ref="R76:R78"/>
+    <mergeCell ref="S76:S78"/>
+    <mergeCell ref="R68:R70"/>
+    <mergeCell ref="S68:S70"/>
+    <mergeCell ref="R64:R66"/>
+    <mergeCell ref="S64:S66"/>
+    <mergeCell ref="S5:S10"/>
+    <mergeCell ref="S12:S14"/>
+    <mergeCell ref="R16:R18"/>
+    <mergeCell ref="R12:R14"/>
+    <mergeCell ref="S16:S18"/>
+    <mergeCell ref="R5:R9"/>
+    <mergeCell ref="C27:C30"/>
+    <mergeCell ref="R48:R50"/>
+    <mergeCell ref="S48:S50"/>
+    <mergeCell ref="R44:R46"/>
+    <mergeCell ref="S44:S46"/>
+    <mergeCell ref="R40:R42"/>
+    <mergeCell ref="S40:S42"/>
+    <mergeCell ref="E31:E34"/>
+    <mergeCell ref="F31:F34"/>
     <mergeCell ref="R32:R34"/>
     <mergeCell ref="S32:S34"/>
-    <mergeCell ref="E23:E26"/>
-    <mergeCell ref="F23:F26"/>
-    <mergeCell ref="R24:R26"/>
-    <mergeCell ref="S24:S26"/>
+    <mergeCell ref="F27:F30"/>
     <mergeCell ref="E27:E30"/>
-    <mergeCell ref="F27:F30"/>
-    <mergeCell ref="R28:R30"/>
-    <mergeCell ref="S28:S30"/>
-    <mergeCell ref="R64:R66"/>
-    <mergeCell ref="S64:S66"/>
-    <mergeCell ref="R76:R78"/>
-    <mergeCell ref="S76:S78"/>
-    <mergeCell ref="C5:C10"/>
-    <mergeCell ref="F11:F14"/>
-    <mergeCell ref="D5:D10"/>
-    <mergeCell ref="C15:C18"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="E5:E10"/>
-    <mergeCell ref="F15:F18"/>
-    <mergeCell ref="F5:F10"/>
-    <mergeCell ref="E19:E22"/>
-    <mergeCell ref="E11:E14"/>
-    <mergeCell ref="E15:E18"/>
-    <mergeCell ref="F19:F22"/>
+    <mergeCell ref="R36:R38"/>
+    <mergeCell ref="S36:S38"/>
+    <mergeCell ref="F35:F38"/>
     <mergeCell ref="M5:Q6"/>
     <mergeCell ref="G5:L6"/>
     <mergeCell ref="G7:G9"/>
@@ -5110,40 +4943,32 @@
     <mergeCell ref="M7:Q7"/>
     <mergeCell ref="M8:M9"/>
     <mergeCell ref="N8:N9"/>
-    <mergeCell ref="C31:C34"/>
-    <mergeCell ref="R52:R54"/>
-    <mergeCell ref="S52:S54"/>
-    <mergeCell ref="R48:R50"/>
-    <mergeCell ref="S48:S50"/>
-    <mergeCell ref="R44:R46"/>
-    <mergeCell ref="S44:S46"/>
-    <mergeCell ref="E35:E38"/>
-    <mergeCell ref="F35:F38"/>
-    <mergeCell ref="R36:R38"/>
-    <mergeCell ref="S36:S38"/>
-    <mergeCell ref="F31:F34"/>
-    <mergeCell ref="E31:E34"/>
-    <mergeCell ref="R40:R42"/>
-    <mergeCell ref="S40:S42"/>
-    <mergeCell ref="F39:F42"/>
-    <mergeCell ref="S5:S10"/>
+    <mergeCell ref="C5:C10"/>
+    <mergeCell ref="F11:F14"/>
+    <mergeCell ref="D5:D10"/>
+    <mergeCell ref="C15:C18"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="E5:E10"/>
+    <mergeCell ref="F15:F18"/>
+    <mergeCell ref="F5:F10"/>
+    <mergeCell ref="E11:E14"/>
+    <mergeCell ref="E15:E18"/>
+    <mergeCell ref="R80:R82"/>
+    <mergeCell ref="S80:S82"/>
+    <mergeCell ref="R28:R30"/>
+    <mergeCell ref="S28:S30"/>
+    <mergeCell ref="E19:E22"/>
+    <mergeCell ref="F19:F22"/>
+    <mergeCell ref="R20:R22"/>
     <mergeCell ref="S20:S22"/>
-    <mergeCell ref="S12:S14"/>
-    <mergeCell ref="R16:R18"/>
-    <mergeCell ref="R12:R14"/>
-    <mergeCell ref="S16:S18"/>
-    <mergeCell ref="R5:R9"/>
-    <mergeCell ref="R20:R22"/>
+    <mergeCell ref="E23:E26"/>
+    <mergeCell ref="F23:F26"/>
+    <mergeCell ref="R24:R26"/>
+    <mergeCell ref="S24:S26"/>
     <mergeCell ref="R60:R62"/>
     <mergeCell ref="S60:S62"/>
-    <mergeCell ref="S56:S58"/>
-    <mergeCell ref="R56:R58"/>
-    <mergeCell ref="R80:R82"/>
-    <mergeCell ref="S80:S82"/>
     <mergeCell ref="R72:R74"/>
     <mergeCell ref="S72:S74"/>
-    <mergeCell ref="R68:R70"/>
-    <mergeCell ref="S68:S70"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.15748031496062992" bottom="0" header="0" footer="0"/>

</xml_diff>